<commit_message>
并入新网赚，但是注意： WaterSort/Assets/WZ/Firebase/Plugins/x86_64/FirebaseCppApp-12_10_0.bundle WaterSort/Assets/WZ/Firebase/Plugins/x86_64/FirebaseCppApp-12_10_0.so 两者超过了100MB，因此不上传（忽略）
</commit_message>
<xml_diff>
--- a/DesignerConfigs/Datas/Guides.xlsx
+++ b/DesignerConfigs/Datas/Guides.xlsx
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="53">
   <si>
     <t>##var</t>
   </si>
@@ -286,36 +286,6 @@
   </si>
   <si>
     <t>handC:FALSE</t>
-  </si>
-  <si>
-    <t>兑现引导1</t>
-  </si>
-  <si>
-    <t>18,Plane/Plane1/BottomPart/WithdrawBtn/GuidePos</t>
-  </si>
-  <si>
-    <t>18,Plane/Plane1/BottomPart/WithdrawBtn</t>
-  </si>
-  <si>
-    <t>canWithdraw:1,</t>
-  </si>
-  <si>
-    <t>iac:0</t>
-  </si>
-  <si>
-    <t>兑现引导2</t>
-  </si>
-  <si>
-    <t>canWithdraw:1</t>
-  </si>
-  <si>
-    <t>兑现引导3</t>
-  </si>
-  <si>
-    <t>canWithdraw:1;iac:0</t>
-  </si>
-  <si>
-    <t>兑现引导4</t>
   </si>
 </sst>
 </file>
@@ -1778,152 +1748,56 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" ht="27" spans="1:18">
-      <c r="B11">
-        <v>10006</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E11">
-        <v>10006</v>
-      </c>
-      <c r="F11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" t="b">
-        <v>1</v>
-      </c>
+    <row r="11" spans="1:18">
+      <c r="D11" s="7"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
       <c r="K11" s="6"/>
-      <c r="L11" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="M11" t="b">
-        <v>1</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="O11" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="L11" s="6"/>
+      <c r="M11"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
       <c r="P11" s="6"/>
-      <c r="Q11" t="s">
-        <v>56</v>
-      </c>
-      <c r="R11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" ht="27" spans="1:18">
-      <c r="B12">
-        <v>10007</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12">
-        <v>10007</v>
-      </c>
-      <c r="F12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" t="b">
-        <v>1</v>
-      </c>
+    </row>
+    <row r="12" spans="1:18">
+      <c r="D12" s="8"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
       <c r="K12" s="6"/>
-      <c r="L12" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="M12" t="b">
-        <v>1</v>
-      </c>
-      <c r="N12" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="O12" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="L12" s="6"/>
+      <c r="M12"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
       <c r="P12" s="6"/>
-      <c r="Q12" t="s">
-        <v>59</v>
-      </c>
-      <c r="R12" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" customFormat="1" ht="27" spans="1:18">
-      <c r="B13">
-        <v>10008</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="E13">
-        <v>10008</v>
-      </c>
-      <c r="F13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" t="b">
-        <v>0</v>
-      </c>
+    </row>
+    <row r="13" customFormat="1" spans="1:18">
+      <c r="D13" s="7"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13"/>
       <c r="H13"/>
       <c r="K13" s="6"/>
-      <c r="L13" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="M13" t="b">
-        <v>1</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="O13" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="L13" s="6"/>
+      <c r="M13"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
       <c r="P13" s="6"/>
-      <c r="Q13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" s="1" customFormat="1" ht="27" spans="1:18">
-      <c r="B14">
-        <v>10009</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="E14">
-        <v>10009</v>
-      </c>
-      <c r="F14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G14" t="b">
-        <v>1</v>
-      </c>
+    </row>
+    <row r="14" s="1" customFormat="1" spans="1:18">
+      <c r="B14"/>
+      <c r="D14" s="8"/>
+      <c r="E14"/>
+      <c r="F14"/>
+      <c r="G14"/>
       <c r="H14" s="1"/>
       <c r="K14" s="9"/>
-      <c r="L14" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="M14" t="b">
-        <v>1</v>
-      </c>
-      <c r="N14" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="O14" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="L14" s="6"/>
+      <c r="M14"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
       <c r="P14" s="9"/>
-      <c r="Q14" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="R14" s="1" t="s">
-        <v>57</v>
-      </c>
     </row>
     <row r="15" customFormat="1" spans="1:18">
       <c r="D15" s="7"/>

</xml_diff>